<commit_message>
WIP snapshot: Levels 2-4 lessons still in review (not final)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GVxwagJ2ocBAdfHuqZnXCC
</commit_message>
<xml_diff>
--- a/02-formulas-functions/01-logical-functions/2.1-logical-functions.xlsx
+++ b/02-formulas-functions/01-logical-functions/2.1-logical-functions.xlsx
@@ -1037,10 +1037,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="64" customHeight="1">
+    <row r="2" ht="79" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>Tasks 1–3 use the Labs sheet. Tasks 4–13 use the ED sheet. Several tasks ask you to fill one of the yellow columns on a data sheet: type the formula in the first data row and Excel fills the rest of the Table column for you (if it doesn't, double-click the fill handle). The gray cell on this sheet then summarizes your column. When a formula on this sheet points at a data sheet, include the sheet name (for example Labs!E38), or click the cell on that sheet and Excel adds the name for you.</t>
+          <t>Tasks 1–3 use the Labs sheet. Tasks 4–13 use the ED sheet. Several tasks ask you to fill one of the yellow columns on a data sheet: type the formula in the first data row and Excel fills the rest of the Table column for you (if it doesn't, double-click the fill handle). The gray cell on this sheet then summarizes your column. When a formula on this sheet points at a data sheet, include the sheet name (for example Labs!E2), or click the cell on that sheet and Excel adds the name for you. Tasks 4 and 11 use IFS and SWITCH, which need Excel 2019 or later. In Excel 2016 or earlier, build those two columns with nested IFs instead. The gray cells count the labels, so the checks still work.</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       </c>
       <c r="C15" s="20" t="inlineStr">
         <is>
-          <t>COUNTIF with a "&gt;=2" criterion</t>
+          <t>COUNTIF with "&gt;=2" as the criteria</t>
         </is>
       </c>
       <c r="D15" s="21" t="n"/>
@@ -1349,7 +1349,7 @@
       </c>
       <c r="B17" s="19" t="inlineStr">
         <is>
-          <t>Shock index = HeartRate ÷ SystolicBP, and 1.0 or more is a warning sign. Fill the yellow ShockIndex column, wrapping the division in IFERROR so the 12 visits with no SystolicBP show a blank ("") instead of #DIV/0!. Start in Q2. The gray cell counts visits with a shock index of 1.0 or higher (it asks you to fix any errors first).</t>
+          <t>Shock index = HeartRate ÷ SystolicBP, and 1.0 or more is a warning sign. Fill the yellow ShockIndex column, wrapping the division in IFERROR so the 12 visits with no SystolicBP show a blank ("") instead of #DIV/0!. Start in Q2. The gray cell counts visits with a shock index of 1.0 or higher. While any #DIV/0! errors are left in your column, it shows "Fix the errors first" instead.</t>
         </is>
       </c>
       <c r="C17" s="20" t="inlineStr">
@@ -39296,7 +39296,7 @@
       </c>
       <c r="B6" s="19" t="inlineStr">
         <is>
-          <t>Fill the qSOFA column (0–3) on the ED sheet, starting in R2. The gray cell adds up your whole column. What is the total number of qSOFA points?</t>
+          <t>Fill the yellow qSOFA column with a score from 0 to 3 on the ED sheet, starting in R2. The gray cell adds up your whole column, so it shows the total number of qSOFA points.</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
@@ -39513,7 +39513,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="96" customHeight="1">
+    <row r="6" ht="126" customHeight="1">
       <c r="A6" s="18" t="inlineStr">
         <is>
           <t>2</t>
@@ -39538,7 +39538,7 @@
       </c>
       <c r="F6" s="19" t="inlineStr">
         <is>
-          <t>Comparing two ranges row by row gives a list of TRUE/FALSE values. The double minus (--) converts them to 1s and 0s, and SUMPRODUCT adds them. In Microsoft 365 and Excel 2021 or later, =SUM(--(…&gt;…)) works too. Plain SUM over a column of TRUE/FALSE *cells* returns 0, because SUM ignores logical values stored in cells.</t>
+          <t>Comparing two ranges row by row gives a list of TRUE/FALSE values. The double minus (--) converts them to 1s and 0s, and SUMPRODUCT adds them. In Microsoft 365 and Excel 2021 or later, =SUM(--(…&gt;…)) works too. COUNTIF can't do this, because it compares one range with one fixed criteria, and here every row has its own RefHigh. Plain SUM over a column of TRUE/FALSE *cells* returns 0, because SUM ignores logical values stored in cells.</t>
         </is>
       </c>
     </row>
@@ -39745,7 +39745,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="66" customHeight="1">
+    <row r="14" ht="96" customHeight="1">
       <c r="A14" s="18" t="inlineStr">
         <is>
           <t>10</t>
@@ -39770,7 +39770,7 @@
       </c>
       <c r="F14" s="19" t="inlineStr">
         <is>
-          <t>Once the score is a number, COUNTIF can count any threshold. The key's live formula does the whole thing in one cell: it builds the score for every row as an array, then counts the rows where it is &gt;=2.</t>
+          <t>Once the score is a number, COUNTIF can count any threshold. The criteria "&gt;=2" keeps the operator and the number together inside one pair of quotes. =SUMPRODUCT(--(ED!O2:O424&gt;=2)) gives the same answer. The key's live formula does the whole thing in one cell: it builds the score for every row as an array, then counts the rows where it is &gt;=2.</t>
         </is>
       </c>
     </row>
@@ -39811,7 +39811,7 @@
       </c>
       <c r="B16" s="19" t="inlineStr">
         <is>
-          <t>Shock index = HeartRate ÷ SystolicBP, and 1.0 or more is a warning sign. Fill the yellow ShockIndex column, wrapping the division in IFERROR so the 12 visits with no SystolicBP show a blank ("") instead of #DIV/0!. Start in Q2. The gray cell counts visits with a shock index of 1.0 or higher (it asks you to fix any errors first).</t>
+          <t>Shock index = HeartRate ÷ SystolicBP, and 1.0 or more is a warning sign. Fill the yellow ShockIndex column, wrapping the division in IFERROR so the 12 visits with no SystolicBP show a blank ("") instead of #DIV/0!. Start in Q2. The gray cell counts visits with a shock index of 1.0 or higher. While any #DIV/0! errors are left in your column, it shows "Fix the errors first" instead.</t>
         </is>
       </c>
       <c r="C16" s="34" t="n">
@@ -39828,7 +39828,7 @@
       </c>
       <c r="F16" s="19" t="inlineStr">
         <is>
-          <t>Dividing by an empty cell divides by zero, so those rows show #DIV/0!. IFERROR(G2/I2,"") returns the division when it works and an empty text string when it fails. COUNTIF then skips the blanks because they are text. =IF(I2="","",G2/I2) is an even better formula, because it handles the one problem you expect (a missing BP) and still lets any *other* mistake show up as an error.</t>
+          <t>Dividing by an empty cell divides by zero, so those rows show #DIV/0!. IFERROR(G2/I2,"") returns the division when it works and empty text when it fails. COUNTIF then skips the blanks because they are text. =IF(I2="","",G2/I2) is an even better formula, because it handles the one problem you expect (a missing BP) and still lets any *other* mistake show up as an error.</t>
         </is>
       </c>
     </row>
@@ -39945,7 +39945,7 @@
       </c>
       <c r="B5" s="19" t="inlineStr">
         <is>
-          <t>Fill the qSOFA column (0–3) on the ED sheet, starting in R2. The gray cell adds up your whole column. What is the total number of qSOFA points?</t>
+          <t>Fill the yellow qSOFA column with a score from 0 to 3 on the ED sheet, starting in R2. The gray cell adds up your whole column, so it shows the total number of qSOFA points.</t>
         </is>
       </c>
       <c r="C5" s="34" t="n">

</xml_diff>